<commit_message>
feat: add new analysis and EIMSA spreadsheets to project documentation
</commit_message>
<xml_diff>
--- a/OI/a2_trs/TP analyse centre usinage.xlsx
+++ b/OI/a2_trs/TP analyse centre usinage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/A2 TRS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/a2_trs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{FBACCD43-1F08-4960-A2F5-622601195D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CF7664F-A2D2-4A6C-AF5E-ADCAB5E0AD38}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="13_ncr:1_{FBACCD43-1F08-4960-A2F5-622601195D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{925C6652-CF0B-4F02-B836-38B8D0EDACBE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B317174-6610-4FA1-8F85-0AE134DA76FE}"/>
+    <workbookView xWindow="14335" yWindow="-65" windowWidth="19330" windowHeight="10210" activeTab="1" xr2:uid="{0B317174-6610-4FA1-8F85-0AE134DA76FE}"/>
   </bookViews>
   <sheets>
     <sheet name="TRS" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="97">
   <si>
     <t>Quantité produite  par C31</t>
   </si>
@@ -55,9 +55,6 @@
     <t>Quantité acceptée C41</t>
   </si>
   <si>
-    <t>Temps d'ouverture</t>
-  </si>
-  <si>
     <t>Quantité totale acceptée</t>
   </si>
   <si>
@@ -317,13 +314,25 @@
   </si>
   <si>
     <t>Travail à faire : Voir les deux onglets</t>
+  </si>
+  <si>
+    <t>Temps d'ouverture TO=TR</t>
+  </si>
+  <si>
+    <t>TRS = TxQ.TxPerf.Do</t>
+  </si>
+  <si>
+    <t>TRS Mensuel =</t>
+  </si>
+  <si>
+    <t>TRS réel =</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -359,6 +368,21 @@
       <b/>
       <sz val="16"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -414,7 +438,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -437,11 +461,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -492,7 +528,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -514,9 +549,29 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -529,6 +584,1592 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>TRS</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>TRS!$B$28:$W$28</c:f>
+              <c:numCache>
+                <c:formatCode>d\-mmm</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>44166</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>44167</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44170</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44171</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44172</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>44173</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>44174</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44177</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44178</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>44179</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>44180</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>44181</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>44184</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>44185</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>44186</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>44187</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>44188</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>44191</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>44192</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>44193</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>44194</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>44195</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>TRS!$B$39:$W$39</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0" formatCode="0.00%">
+                  <c:v>0.58139534883720922</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.86794019933554811</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.89285714285714279</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.35299003322259137</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.95514950166112955</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.78903654485049834</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.88870431893687707</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.59800664451827235</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.72259136212624586</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.59385382059800662</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.97176079734219267</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.87624584717607967</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.98421926910298996</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.58970099667774079</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.88039867109634551</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.47757475083056478</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.71843853820598003</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.95930232558139528</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.59385382059800662</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-38DC-4684-85E5-1ED2A6560E94}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>TxQ</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>TRS!$B$28:$W$28</c:f>
+              <c:numCache>
+                <c:formatCode>d\-mmm</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>44166</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>44167</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44170</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44171</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44172</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>44173</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>44174</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44177</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44178</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>44179</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>44180</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>44181</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>44184</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>44185</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>44186</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>44187</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>44188</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>44191</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>44192</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>44193</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>44194</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>44195</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>TRS!$B$40:$W$40</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0" formatCode="0.00%">
+                  <c:v>0.97902097902097907</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.95871559633027525</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.99537037037037035</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.97701149425287359</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.97046413502109707</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.97272727272727277</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.97959183673469385</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.98305084745762716</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.99152542372881358</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.99061032863849763</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.98611111111111116</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.99530516431924887</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.98857142857142855</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.99568965517241381</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.98620689655172411</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-38DC-4684-85E5-1ED2A6560E94}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>TxPerf</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>TRS!$B$28:$W$28</c:f>
+              <c:numCache>
+                <c:formatCode>d\-mmm</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>44166</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>44167</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44170</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44171</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44172</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>44173</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>44174</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44177</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44178</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>44179</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>44180</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>44181</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>44184</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>44185</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>44186</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>44187</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>44188</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>44191</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>44192</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>44193</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>44194</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>44195</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>TRS!$B$41:$W$41</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0" formatCode="0.00%">
+                  <c:v>0.95016611295681064</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.96566998892580291</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.95681063122923582</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.96345514950166111</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.98421926910298996</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.97112190135445953</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.9745293466223699</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.97674418604651159</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.98006644518272423</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.86378737541528239</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.98006644518272423</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.94352159468438535</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.98421926910298996</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.95681063122923571</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.88455149501661123</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.95514950166112955</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.96899224806201545</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.96345514950166111</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.96345514950166111</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-38DC-4684-85E5-1ED2A6560E94}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>DO</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>TRS!$B$28:$W$28</c:f>
+              <c:numCache>
+                <c:formatCode>d\-mmm</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>44166</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>44167</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44170</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44171</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44172</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>44173</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>44174</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44177</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44178</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>44179</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>44180</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>44181</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>44184</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>44185</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>44186</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>44187</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>44188</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>44191</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>44192</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>44193</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>44194</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>44195</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>TRS!$B$42:$W$42</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0" formatCode="0.00%">
+                  <c:v>0.625</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.9375</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.9375</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.375</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.8125</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.9375</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.625</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.6875</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.9375</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.625</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.625</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-38DC-4684-85E5-1ED2A6560E94}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="378411744"/>
+        <c:axId val="577329728"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="378411744"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="44196"/>
+          <c:min val="44166"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="d\-mmm" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="577329728"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="1"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="577329728"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="378411744"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>236467</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>103118</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>513521</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>122514</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Graphique 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3806B0B-816A-F26C-409E-283485612ABD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -828,160 +2469,161 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{360368A5-3BBC-48BD-A4CF-04033307A40A}">
-  <dimension ref="A1:W42"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:X46"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="23" width="7.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.53125" customWidth="1"/>
+    <col min="3" max="23" width="7.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
-        <v>93</v>
-      </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="24"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A3" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A4" s="23"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
+    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B16" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
       <c r="H16" s="19">
         <v>15.7</v>
       </c>
       <c r="I16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="B17" s="24" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B17" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
       <c r="H17" s="19">
         <v>14.4</v>
       </c>
       <c r="I17" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.45">
       <c r="B18" s="9"/>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.45">
       <c r="B19" s="9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.45">
       <c r="B20" s="9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.45">
       <c r="B21" s="9"/>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.45">
       <c r="B22" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.45">
       <c r="B23" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.45">
       <c r="B24" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="B25" s="9" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B25" s="9" t="s">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="B26" s="9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B26" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A28" s="2"/>
       <c r="B28" s="5">
         <v>44166</v>
@@ -1050,9 +2692,9 @@
         <v>44195</v>
       </c>
     </row>
-    <row r="29" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>6</v>
+        <v>93</v>
       </c>
       <c r="B29" s="6">
         <v>8</v>
@@ -1121,9 +2763,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B30" s="6">
         <v>3</v>
@@ -1192,61 +2834,197 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
-      <c r="I31" s="21"/>
-      <c r="J31" s="21"/>
-      <c r="K31" s="21"/>
-      <c r="L31" s="21"/>
-      <c r="M31" s="21"/>
-      <c r="N31" s="21"/>
-      <c r="O31" s="21"/>
-      <c r="P31" s="21"/>
-      <c r="Q31" s="21"/>
-      <c r="R31" s="21"/>
-      <c r="S31" s="21"/>
-      <c r="T31" s="21"/>
-      <c r="U31" s="21"/>
-      <c r="V31" s="21"/>
-      <c r="W31" s="21"/>
-    </row>
-    <row r="32" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="B31" s="21">
+        <f>B29-B30</f>
+        <v>5</v>
+      </c>
+      <c r="C31" s="21">
+        <f t="shared" ref="C31:W31" si="0">C29-C30</f>
+        <v>7.5</v>
+      </c>
+      <c r="D31" s="21">
+        <f t="shared" si="0"/>
+        <v>7.5</v>
+      </c>
+      <c r="E31" s="21">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="F31" s="21">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="G31" s="21">
+        <f t="shared" si="0"/>
+        <v>6.5</v>
+      </c>
+      <c r="H31" s="21">
+        <f t="shared" si="0"/>
+        <v>7.5</v>
+      </c>
+      <c r="I31" s="21">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="J31" s="21">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="K31" s="21">
+        <f t="shared" si="0"/>
+        <v>5.5</v>
+      </c>
+      <c r="L31" s="21">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="M31" s="21">
+        <f t="shared" si="0"/>
+        <v>7.5</v>
+      </c>
+      <c r="N31" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O31" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P31" s="21">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="Q31" s="21">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="R31" s="21">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="S31" s="21">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="T31" s="21">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="U31" s="21">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="V31" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W31" s="21">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B32" s="21"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21"/>
-      <c r="L32" s="21"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="21"/>
-      <c r="O32" s="21"/>
-      <c r="P32" s="21"/>
-      <c r="Q32" s="21"/>
-      <c r="R32" s="21"/>
-      <c r="S32" s="21"/>
-      <c r="T32" s="21"/>
-      <c r="U32" s="21"/>
-      <c r="V32" s="21"/>
-      <c r="W32" s="21"/>
-    </row>
-    <row r="33" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="21">
+        <f>B29*15.7+B29*14.4</f>
+        <v>240.8</v>
+      </c>
+      <c r="C32" s="21">
+        <f t="shared" ref="C32:W32" si="1">C29*15.7+C29*14.4</f>
+        <v>240.8</v>
+      </c>
+      <c r="D32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="E32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="F32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="G32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="H32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="I32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="J32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="K32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="L32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="M32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="N32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="O32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="P32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="Q32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="R32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="S32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="T32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="U32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="V32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="W32" s="21">
+        <f t="shared" si="1"/>
+        <v>240.8</v>
+      </c>
+      <c r="X32" s="1">
+        <f>SUM(B32:W32)</f>
+        <v>5297.6000000000022</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="4" t="s">
         <v>0</v>
       </c>
@@ -1317,7 +3095,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="34" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="4" t="s">
         <v>1</v>
       </c>
@@ -1388,34 +3166,100 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B35" s="21"/>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-      <c r="G35" s="21"/>
-      <c r="H35" s="21"/>
-      <c r="I35" s="21"/>
-      <c r="J35" s="21"/>
-      <c r="K35" s="21"/>
-      <c r="L35" s="21"/>
-      <c r="M35" s="21"/>
-      <c r="N35" s="21"/>
-      <c r="O35" s="21"/>
-      <c r="P35" s="21"/>
-      <c r="Q35" s="21"/>
-      <c r="R35" s="21"/>
-      <c r="S35" s="21"/>
-      <c r="T35" s="21"/>
-      <c r="U35" s="21"/>
-      <c r="V35" s="21"/>
-      <c r="W35" s="21"/>
-    </row>
-    <row r="36" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="21">
+        <f>B33+B34</f>
+        <v>143</v>
+      </c>
+      <c r="C35" s="21">
+        <f t="shared" ref="C35:W35" si="2">C33+C34</f>
+        <v>218</v>
+      </c>
+      <c r="D35" s="21">
+        <f t="shared" si="2"/>
+        <v>216</v>
+      </c>
+      <c r="E35" s="21">
+        <f t="shared" si="2"/>
+        <v>87</v>
+      </c>
+      <c r="F35" s="21">
+        <f t="shared" si="2"/>
+        <v>237</v>
+      </c>
+      <c r="G35" s="21">
+        <f t="shared" si="2"/>
+        <v>190</v>
+      </c>
+      <c r="H35" s="21">
+        <f t="shared" si="2"/>
+        <v>220</v>
+      </c>
+      <c r="I35" s="21">
+        <f t="shared" si="2"/>
+        <v>147</v>
+      </c>
+      <c r="J35" s="21">
+        <f t="shared" si="2"/>
+        <v>177</v>
+      </c>
+      <c r="K35" s="21">
+        <f t="shared" si="2"/>
+        <v>143</v>
+      </c>
+      <c r="L35" s="21">
+        <f t="shared" si="2"/>
+        <v>236</v>
+      </c>
+      <c r="M35" s="21">
+        <f t="shared" si="2"/>
+        <v>213</v>
+      </c>
+      <c r="N35" s="21">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O35" s="21">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P35" s="21">
+        <f t="shared" si="2"/>
+        <v>237</v>
+      </c>
+      <c r="Q35" s="21">
+        <f t="shared" si="2"/>
+        <v>144</v>
+      </c>
+      <c r="R35" s="21">
+        <f t="shared" si="2"/>
+        <v>213</v>
+      </c>
+      <c r="S35" s="21">
+        <f t="shared" si="2"/>
+        <v>115</v>
+      </c>
+      <c r="T35" s="21">
+        <f t="shared" si="2"/>
+        <v>175</v>
+      </c>
+      <c r="U35" s="21">
+        <f t="shared" si="2"/>
+        <v>232</v>
+      </c>
+      <c r="V35" s="21">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W35" s="21">
+        <f t="shared" si="2"/>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="4" t="s">
         <v>4</v>
       </c>
@@ -1486,7 +3330,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="37" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="4" t="s">
         <v>5</v>
       </c>
@@ -1557,140 +3401,589 @@
         <v>67</v>
       </c>
     </row>
-    <row r="38" spans="1:23" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:24" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38" s="21">
+        <f>B36+B37</f>
+        <v>140</v>
+      </c>
+      <c r="C38" s="21">
+        <f t="shared" ref="C38:W38" si="3">C36+C37</f>
+        <v>209</v>
+      </c>
+      <c r="D38" s="21">
+        <f t="shared" si="3"/>
+        <v>215</v>
+      </c>
+      <c r="E38" s="21">
+        <f t="shared" si="3"/>
+        <v>85</v>
+      </c>
+      <c r="F38" s="21">
+        <f t="shared" si="3"/>
+        <v>230</v>
+      </c>
+      <c r="G38" s="21">
+        <f t="shared" si="3"/>
+        <v>190</v>
+      </c>
+      <c r="H38" s="21">
+        <f t="shared" si="3"/>
+        <v>214</v>
+      </c>
+      <c r="I38" s="21">
+        <f t="shared" si="3"/>
+        <v>144</v>
+      </c>
+      <c r="J38" s="21">
+        <f t="shared" si="3"/>
+        <v>174</v>
+      </c>
+      <c r="K38" s="21">
+        <f t="shared" si="3"/>
+        <v>143</v>
+      </c>
+      <c r="L38" s="21">
+        <f t="shared" si="3"/>
+        <v>234</v>
+      </c>
+      <c r="M38" s="21">
+        <f t="shared" si="3"/>
+        <v>211</v>
+      </c>
+      <c r="N38" s="21">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O38" s="21">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="P38" s="21">
+        <f t="shared" si="3"/>
+        <v>237</v>
+      </c>
+      <c r="Q38" s="21">
+        <f t="shared" si="3"/>
+        <v>142</v>
+      </c>
+      <c r="R38" s="21">
+        <f t="shared" si="3"/>
+        <v>212</v>
+      </c>
+      <c r="S38" s="21">
+        <f t="shared" si="3"/>
+        <v>115</v>
+      </c>
+      <c r="T38" s="21">
+        <f t="shared" si="3"/>
+        <v>173</v>
+      </c>
+      <c r="U38" s="21">
+        <f t="shared" si="3"/>
+        <v>231</v>
+      </c>
+      <c r="V38" s="21">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="W38" s="21">
+        <f t="shared" si="3"/>
+        <v>143</v>
+      </c>
+      <c r="X38" s="1">
+        <f>SUM(B38:W38)</f>
+        <v>3442</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A39" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B38" s="21"/>
-      <c r="C38" s="21"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="21"/>
-      <c r="F38" s="21"/>
-      <c r="G38" s="21"/>
-      <c r="H38" s="21"/>
-      <c r="I38" s="21"/>
-      <c r="J38" s="21"/>
-      <c r="K38" s="21"/>
-      <c r="L38" s="21"/>
-      <c r="M38" s="21"/>
-      <c r="N38" s="21"/>
-      <c r="O38" s="21"/>
-      <c r="P38" s="21"/>
-      <c r="Q38" s="21"/>
-      <c r="R38" s="21"/>
-      <c r="S38" s="21"/>
-      <c r="T38" s="21"/>
-      <c r="U38" s="21"/>
-      <c r="V38" s="21"/>
-      <c r="W38" s="21"/>
-    </row>
-    <row r="39" spans="1:23" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="8"/>
-      <c r="K39" s="8"/>
-      <c r="L39" s="8"/>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
-      <c r="P39" s="8"/>
-      <c r="Q39" s="8"/>
-      <c r="R39" s="8"/>
-      <c r="S39" s="8"/>
-      <c r="T39" s="8"/>
-      <c r="U39" s="8"/>
-      <c r="V39" s="8"/>
-      <c r="W39" s="8"/>
-    </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B39" s="33">
+        <f>B38/B32</f>
+        <v>0.58139534883720922</v>
+      </c>
+      <c r="C39" s="30">
+        <f t="shared" ref="C39:W39" si="4">C38/C32</f>
+        <v>0.86794019933554811</v>
+      </c>
+      <c r="D39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.89285714285714279</v>
+      </c>
+      <c r="E39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.35299003322259137</v>
+      </c>
+      <c r="F39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.95514950166112955</v>
+      </c>
+      <c r="G39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.78903654485049834</v>
+      </c>
+      <c r="H39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.88870431893687707</v>
+      </c>
+      <c r="I39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.59800664451827235</v>
+      </c>
+      <c r="J39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.72259136212624586</v>
+      </c>
+      <c r="K39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.59385382059800662</v>
+      </c>
+      <c r="L39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.97176079734219267</v>
+      </c>
+      <c r="M39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.87624584717607967</v>
+      </c>
+      <c r="N39" s="30">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="O39" s="30">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.98421926910298996</v>
+      </c>
+      <c r="Q39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.58970099667774079</v>
+      </c>
+      <c r="R39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.88039867109634551</v>
+      </c>
+      <c r="S39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.47757475083056478</v>
+      </c>
+      <c r="T39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.71843853820598003</v>
+      </c>
+      <c r="U39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.95930232558139528</v>
+      </c>
+      <c r="V39" s="30">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="W39" s="30">
+        <f t="shared" si="4"/>
+        <v>0.59385382059800662</v>
+      </c>
+      <c r="X39" s="37">
+        <f>AVERAGE(B39:W39)</f>
+        <v>0.6497281787979462</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A40" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="B40" s="34">
+        <f>B38/B35</f>
+        <v>0.97902097902097907</v>
+      </c>
+      <c r="C40" s="29">
+        <f t="shared" ref="C40:W40" si="5">C38/C35</f>
+        <v>0.95871559633027525</v>
+      </c>
+      <c r="D40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.99537037037037035</v>
+      </c>
+      <c r="E40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.97701149425287359</v>
+      </c>
+      <c r="F40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.97046413502109707</v>
+      </c>
+      <c r="G40" s="29">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="H40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.97272727272727277</v>
+      </c>
+      <c r="I40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.97959183673469385</v>
+      </c>
+      <c r="J40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.98305084745762716</v>
+      </c>
+      <c r="K40" s="29">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="L40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.99152542372881358</v>
+      </c>
+      <c r="M40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.99061032863849763</v>
+      </c>
+      <c r="N40" s="29" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="O40" s="29" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="P40" s="29">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="Q40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="R40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.99530516431924887</v>
+      </c>
+      <c r="S40" s="29">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="T40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.98857142857142855</v>
+      </c>
+      <c r="U40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.99568965517241381</v>
+      </c>
+      <c r="V40" s="29" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W40" s="29">
+        <f t="shared" si="5"/>
+        <v>0.98620689655172411</v>
+      </c>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A41" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="B40" s="22"/>
-      <c r="C40" s="22"/>
-      <c r="D40" s="22"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
-      <c r="K40" s="22"/>
-      <c r="L40" s="22"/>
-      <c r="M40" s="22"/>
-      <c r="N40" s="22"/>
-      <c r="O40" s="22"/>
-      <c r="P40" s="22"/>
-      <c r="Q40" s="22"/>
-      <c r="R40" s="22"/>
-      <c r="S40" s="22"/>
-      <c r="T40" s="22"/>
-      <c r="U40" s="22"/>
-      <c r="V40" s="22"/>
-      <c r="W40" s="22"/>
-    </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A41" s="20" t="s">
+      <c r="B41" s="34">
+        <f>(B35/30.1)/B31</f>
+        <v>0.95016611295681064</v>
+      </c>
+      <c r="C41" s="29">
+        <f t="shared" ref="C41:W41" si="6">(C35/30.1)/C31</f>
+        <v>0.96566998892580291</v>
+      </c>
+      <c r="D41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.95681063122923582</v>
+      </c>
+      <c r="E41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.96345514950166111</v>
+      </c>
+      <c r="F41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.98421926910298996</v>
+      </c>
+      <c r="G41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.97112190135445953</v>
+      </c>
+      <c r="H41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.9745293466223699</v>
+      </c>
+      <c r="I41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.97674418604651159</v>
+      </c>
+      <c r="J41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.98006644518272423</v>
+      </c>
+      <c r="K41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.86378737541528239</v>
+      </c>
+      <c r="L41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.98006644518272423</v>
+      </c>
+      <c r="M41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.94352159468438535</v>
+      </c>
+      <c r="N41" s="29" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="O41" s="29" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="P41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.98421926910298996</v>
+      </c>
+      <c r="Q41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.95681063122923571</v>
+      </c>
+      <c r="R41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.88455149501661123</v>
+      </c>
+      <c r="S41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.95514950166112955</v>
+      </c>
+      <c r="T41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="U41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.96345514950166111</v>
+      </c>
+      <c r="V41" s="29" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W41" s="29">
+        <f t="shared" si="6"/>
+        <v>0.96345514950166111</v>
+      </c>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A42" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="B41" s="22"/>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
-      <c r="N41" s="22"/>
-      <c r="O41" s="22"/>
-      <c r="P41" s="22"/>
-      <c r="Q41" s="22"/>
-      <c r="R41" s="22"/>
-      <c r="S41" s="22"/>
-      <c r="T41" s="22"/>
-      <c r="U41" s="22"/>
-      <c r="V41" s="22"/>
-      <c r="W41" s="22"/>
-    </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="B42" s="22"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22"/>
-      <c r="I42" s="22"/>
-      <c r="J42" s="22"/>
-      <c r="K42" s="22"/>
-      <c r="L42" s="22"/>
-      <c r="M42" s="22"/>
-      <c r="N42" s="22"/>
-      <c r="O42" s="22"/>
-      <c r="P42" s="22"/>
-      <c r="Q42" s="22"/>
-      <c r="R42" s="22"/>
-      <c r="S42" s="22"/>
-      <c r="T42" s="22"/>
-      <c r="U42" s="22"/>
-      <c r="V42" s="22"/>
-      <c r="W42" s="22"/>
+      <c r="B42" s="34">
+        <f>B31/B29</f>
+        <v>0.625</v>
+      </c>
+      <c r="C42" s="29">
+        <f t="shared" ref="C42:W42" si="7">C31/C29</f>
+        <v>0.9375</v>
+      </c>
+      <c r="D42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.9375</v>
+      </c>
+      <c r="E42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.375</v>
+      </c>
+      <c r="F42" s="29">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="G42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.8125</v>
+      </c>
+      <c r="H42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.9375</v>
+      </c>
+      <c r="I42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.625</v>
+      </c>
+      <c r="J42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.75</v>
+      </c>
+      <c r="K42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.6875</v>
+      </c>
+      <c r="L42" s="29">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="M42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.9375</v>
+      </c>
+      <c r="N42" s="29">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="O42" s="29">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="P42" s="29">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="Q42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.625</v>
+      </c>
+      <c r="R42" s="29">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="S42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.5</v>
+      </c>
+      <c r="T42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.75</v>
+      </c>
+      <c r="U42" s="29">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="V42" s="29">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W42" s="29">
+        <f t="shared" si="7"/>
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A43" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43" s="35">
+        <f>PRODUCT(B40:B42)</f>
+        <v>0.58139534883720934</v>
+      </c>
+      <c r="C43" s="32">
+        <f t="shared" ref="C43:W43" si="8">PRODUCT(C40:C42)</f>
+        <v>0.86794019933554822</v>
+      </c>
+      <c r="D43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.89285714285714279</v>
+      </c>
+      <c r="E43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.35299003322259137</v>
+      </c>
+      <c r="F43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.95514950166112955</v>
+      </c>
+      <c r="G43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.78903654485049834</v>
+      </c>
+      <c r="H43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.88870431893687718</v>
+      </c>
+      <c r="I43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.59800664451827235</v>
+      </c>
+      <c r="J43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.72259136212624586</v>
+      </c>
+      <c r="K43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.59385382059800662</v>
+      </c>
+      <c r="L43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.97176079734219267</v>
+      </c>
+      <c r="M43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.87624584717607967</v>
+      </c>
+      <c r="N43" s="32" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="O43" s="32" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="P43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.98421926910298996</v>
+      </c>
+      <c r="Q43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.58970099667774079</v>
+      </c>
+      <c r="R43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.88039867109634551</v>
+      </c>
+      <c r="S43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.47757475083056478</v>
+      </c>
+      <c r="T43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.71843853820598003</v>
+      </c>
+      <c r="U43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.95930232558139539</v>
+      </c>
+      <c r="V43" s="32" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W43" s="32">
+        <f t="shared" si="8"/>
+        <v>0.59385382059800662</v>
+      </c>
+    </row>
+    <row r="45" spans="1:24" ht="21" x14ac:dyDescent="0.65">
+      <c r="A45" s="36" t="s">
+        <v>95</v>
+      </c>
+      <c r="B45" s="38">
+        <f>X38/X32</f>
+        <v>0.64972817879794598</v>
+      </c>
+    </row>
+    <row r="46" spans="1:24" ht="21" x14ac:dyDescent="0.65">
+      <c r="A46" s="36" t="s">
+        <v>96</v>
+      </c>
+      <c r="B46" s="39">
+        <f>AVERAGE(B39:M39,P39:U39,W39)</f>
+        <v>0.75231683860814824</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1701,97 +3994,98 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D80FA173-BD41-44D7-8C87-F06F15F5F3FB}">
-  <dimension ref="B2:T57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:T58"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="10" width="4.7109375" customWidth="1"/>
+    <col min="2" max="10" width="4.73046875" customWidth="1"/>
     <col min="11" max="11" width="31" customWidth="1"/>
-    <col min="12" max="12" width="9.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="9.265625" customWidth="1"/>
+    <col min="13" max="13" width="11.265625" customWidth="1"/>
     <col min="14" max="14" width="7" customWidth="1"/>
-    <col min="17" max="17" width="29.140625" customWidth="1"/>
+    <col min="17" max="17" width="29.1328125" customWidth="1"/>
     <col min="18" max="18" width="29" customWidth="1"/>
-    <col min="19" max="19" width="24.5703125" customWidth="1"/>
+    <col min="19" max="19" width="24.59765625" customWidth="1"/>
     <col min="20" max="20" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:16" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="B5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+    <row r="8" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B8" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="L8" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="M8" s="28" t="s">
+        <v>32</v>
+      </c>
+      <c r="N8" s="13"/>
+    </row>
+    <row r="9" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B9" s="7" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="L8" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="M8" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="N8" s="13"/>
-    </row>
-    <row r="9" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="7" t="s">
+      <c r="C9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="G9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="I9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="J9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="K9" s="28"/>
-      <c r="L9" s="29"/>
-      <c r="M9" s="29"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="28"/>
+      <c r="M9" s="28"/>
       <c r="N9" s="13"/>
     </row>
-    <row r="10" spans="2:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B10" s="2"/>
       <c r="C10" s="14"/>
       <c r="D10" s="2"/>
@@ -1802,17 +4096,17 @@
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L10" s="2">
         <v>1.5</v>
       </c>
       <c r="M10" s="15"/>
       <c r="P10" s="10" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -1823,7 +4117,7 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L11" s="2">
         <v>1.5</v>
@@ -1832,11 +4126,13 @@
         <v>53</v>
       </c>
       <c r="P11" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B12" s="14"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="B12" s="14">
+        <v>1</v>
+      </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -1846,7 +4142,7 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L12" s="2">
         <v>8</v>
@@ -1855,10 +4151,10 @@
         <v>1296</v>
       </c>
       <c r="P12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B13" s="2"/>
       <c r="C13" s="14"/>
       <c r="D13" s="2"/>
@@ -1869,17 +4165,17 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L13" s="2">
         <v>1.5</v>
       </c>
       <c r="M13" s="15"/>
       <c r="P13" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -1890,7 +4186,7 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L14" s="2">
         <v>3</v>
@@ -1899,10 +4195,10 @@
         <v>38</v>
       </c>
       <c r="P14" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -1913,7 +4209,7 @@
       <c r="I15" s="2"/>
       <c r="J15" s="14"/>
       <c r="K15" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L15" s="2">
         <v>8</v>
@@ -1922,10 +4218,10 @@
         <v>206</v>
       </c>
       <c r="P15" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="14"/>
@@ -1936,7 +4232,7 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L16" s="2">
         <v>1.5</v>
@@ -1945,11 +4241,13 @@
         <v>114</v>
       </c>
       <c r="P16" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B17" s="14"/>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="B17" s="14">
+        <v>1</v>
+      </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -1959,7 +4257,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L17" s="2">
         <v>6</v>
@@ -1968,7 +4266,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -1979,7 +4277,7 @@
       <c r="I18" s="14"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L18" s="2">
         <v>8</v>
@@ -1988,7 +4286,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -1999,7 +4297,7 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L19" s="2">
         <v>5.5</v>
@@ -2008,7 +4306,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="20" spans="2:20" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" ht="28.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -2019,7 +4317,7 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L20" s="2">
         <v>4.5</v>
@@ -2028,23 +4326,25 @@
         <v>267</v>
       </c>
       <c r="P20" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q20" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="Q20" s="16" t="s">
+      <c r="R20" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="R20" s="17" t="s">
+      <c r="S20" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="S20" s="17" t="s">
+      <c r="T20" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="T20" s="17" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B21" s="14"/>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="B21" s="14">
+        <v>1</v>
+      </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -2054,21 +4354,21 @@
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L21" s="2">
         <v>2</v>
       </c>
       <c r="M21" s="15"/>
       <c r="P21" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
       <c r="T21" s="2"/>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B22" s="2"/>
       <c r="C22" s="14"/>
       <c r="D22" s="2"/>
@@ -2079,7 +4379,7 @@
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L22" s="2">
         <v>1</v>
@@ -2088,14 +4388,14 @@
         <v>27</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
       <c r="S22" s="2"/>
       <c r="T22" s="2"/>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -2106,7 +4406,7 @@
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L23" s="2">
         <v>2.5</v>
@@ -2115,15 +4415,17 @@
         <v>191</v>
       </c>
       <c r="P23" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B24" s="14"/>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="B24" s="14">
+        <v>1</v>
+      </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -2133,21 +4435,21 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L24" s="2">
         <v>2</v>
       </c>
       <c r="M24" s="15"/>
       <c r="P24" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
       <c r="T24" s="2"/>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -2158,21 +4460,21 @@
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L25" s="2">
         <v>6.5</v>
       </c>
       <c r="M25" s="15"/>
       <c r="P25" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="Q25" s="2"/>
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
       <c r="T25" s="2"/>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -2183,21 +4485,21 @@
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L26" s="2">
         <v>3</v>
       </c>
       <c r="M26" s="15"/>
       <c r="P26" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="Q26" s="2"/>
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
       <c r="T26" s="2"/>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="14"/>
@@ -2208,21 +4510,21 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L27" s="2">
         <v>1</v>
       </c>
       <c r="M27" s="15"/>
       <c r="P27" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q27" s="2"/>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
       <c r="T27" s="2"/>
     </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B28" s="2"/>
       <c r="C28" s="14"/>
       <c r="D28" s="2"/>
@@ -2233,22 +4535,24 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L28" s="2">
         <v>1</v>
       </c>
       <c r="M28" s="15"/>
       <c r="P28" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
       <c r="T28" s="2"/>
     </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B29" s="14"/>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="B29" s="14">
+        <v>1</v>
+      </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -2258,21 +4562,21 @@
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L29" s="2">
         <v>0.5</v>
       </c>
       <c r="M29" s="15"/>
       <c r="P29" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
       <c r="T29" s="2"/>
     </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -2283,7 +4587,7 @@
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L30" s="2">
         <v>5</v>
@@ -2292,7 +4596,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -2303,7 +4607,7 @@
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L31" s="2">
         <v>4</v>
@@ -2312,7 +4616,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:20" x14ac:dyDescent="0.45">
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -2323,7 +4627,7 @@
       <c r="I32" s="14"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L32" s="2">
         <v>2</v>
@@ -2332,7 +4636,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B33" s="2"/>
       <c r="C33" s="14"/>
       <c r="D33" s="2"/>
@@ -2343,15 +4647,17 @@
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L33" s="2">
         <v>1</v>
       </c>
       <c r="M33" s="15"/>
     </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B34" s="14"/>
+    <row r="34" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B34" s="14">
+        <v>1</v>
+      </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -2361,7 +4667,7 @@
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L34" s="2">
         <v>1</v>
@@ -2370,7 +4676,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -2381,14 +4687,14 @@
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L35" s="2">
         <v>4</v>
       </c>
       <c r="M35" s="15"/>
     </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -2399,14 +4705,14 @@
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L36" s="2">
         <v>0.5</v>
       </c>
       <c r="M36" s="15"/>
     </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -2417,14 +4723,14 @@
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L37" s="2">
         <v>2</v>
       </c>
       <c r="M37" s="15"/>
     </row>
-    <row r="38" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B38" s="2"/>
       <c r="C38" s="14"/>
       <c r="D38" s="2"/>
@@ -2435,15 +4741,17 @@
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L38" s="2">
         <v>0.5</v>
       </c>
       <c r="M38" s="15"/>
     </row>
-    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B39" s="14"/>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B39" s="14">
+        <v>1</v>
+      </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -2453,7 +4761,7 @@
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L39" s="2">
         <v>2.5</v>
@@ -2462,7 +4770,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B40" s="2"/>
       <c r="C40" s="14"/>
       <c r="D40" s="2"/>
@@ -2473,14 +4781,14 @@
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L40" s="2">
         <v>2.5</v>
       </c>
       <c r="M40" s="15"/>
     </row>
-    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -2491,15 +4799,17 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L41" s="2">
         <v>1</v>
       </c>
       <c r="M41" s="15"/>
     </row>
-    <row r="42" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B42" s="14"/>
+    <row r="42" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B42" s="14">
+        <v>1</v>
+      </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -2509,14 +4819,14 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L42" s="2">
         <v>3.5</v>
       </c>
       <c r="M42" s="15"/>
     </row>
-    <row r="43" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -2527,15 +4837,17 @@
       <c r="I43" s="14"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L43" s="2">
         <v>0.5</v>
       </c>
       <c r="M43" s="15"/>
     </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B44" s="14"/>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B44" s="14">
+        <v>1</v>
+      </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
@@ -2545,14 +4857,14 @@
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L44" s="2">
         <v>2.5</v>
       </c>
       <c r="M44" s="15"/>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
@@ -2563,14 +4875,14 @@
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L45" s="2">
         <v>2.5</v>
       </c>
       <c r="M45" s="15"/>
     </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -2581,14 +4893,14 @@
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L46" s="2">
         <v>3</v>
       </c>
       <c r="M46" s="15"/>
     </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="14"/>
@@ -2599,25 +4911,27 @@
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L47" s="2">
         <v>2</v>
       </c>
       <c r="M47" s="15"/>
     </row>
-    <row r="48" spans="2:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
-      <c r="H48" s="14"/>
+      <c r="H48" s="14">
+        <v>1</v>
+      </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L48" s="2">
         <v>4</v>
@@ -2626,8 +4940,10 @@
         <v>191</v>
       </c>
     </row>
-    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B49" s="14"/>
+    <row r="49" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B49" s="14">
+        <v>1</v>
+      </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
@@ -2637,7 +4953,7 @@
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
       <c r="K49" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L49" s="2">
         <v>1.5</v>
@@ -2646,7 +4962,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
@@ -2657,14 +4973,14 @@
       <c r="I50" s="2"/>
       <c r="J50" s="14"/>
       <c r="K50" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L50" s="2">
         <v>4</v>
       </c>
       <c r="M50" s="15"/>
     </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
@@ -2675,32 +4991,34 @@
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="K51" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L51" s="2">
         <v>3</v>
       </c>
       <c r="M51" s="15"/>
     </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
-      <c r="H52" s="14"/>
+      <c r="H52" s="14">
+        <v>1</v>
+      </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L52" s="2">
         <v>1</v>
       </c>
       <c r="M52" s="15"/>
     </row>
-    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
@@ -2711,7 +5029,7 @@
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L53" s="2">
         <v>8</v>
@@ -2720,7 +5038,7 @@
         <v>3296</v>
       </c>
     </row>
-    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
@@ -2731,7 +5049,7 @@
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L54" s="2">
         <v>1</v>
@@ -2740,8 +5058,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B55" s="14"/>
+    <row r="55" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B55" s="14">
+        <v>1</v>
+      </c>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
@@ -2751,14 +5071,14 @@
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L55" s="2">
         <v>4</v>
       </c>
       <c r="M55" s="15"/>
     </row>
-    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B56" s="2"/>
       <c r="C56" s="14"/>
       <c r="D56" s="2"/>
@@ -2769,15 +5089,17 @@
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L56" s="2">
         <v>1</v>
       </c>
       <c r="M56" s="15"/>
     </row>
-    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B57" s="14"/>
+    <row r="57" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B57" s="14">
+        <v>1</v>
+      </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
@@ -2787,13 +5109,51 @@
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
       <c r="K57" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L57" s="2">
         <v>8</v>
       </c>
       <c r="M57" s="2">
         <v>1944</v>
+      </c>
+    </row>
+    <row r="58" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B58">
+        <f>SUMPRODUCT(B10:B57,$L$10:$L$57)</f>
+        <v>41.5</v>
+      </c>
+      <c r="C58">
+        <f t="shared" ref="C58:J58" si="0">SUMPRODUCT(C10:C57,$L$10:$L$57)</f>
+        <v>0</v>
+      </c>
+      <c r="D58">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E58">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G58">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H58">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I58">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>